<commit_message>
Examples: fix three wrong sample facts and the old preview naming
Sheet 05's note about typing đ sat on ngọn núi, which has no đ; the row
is now con đường. Sheet 11's 日 example used 今日, which is not everyday
Mandarin; it is now 明天是我的生日. Sheet 22 said the hamza in ماء sits on a
seat; it stands alone on the line. Comments say Sheet to Anki, not the
preview site.
</commit_message>
<xml_diff>
--- a/examples/sheetcards-examples.xlsx
+++ b/examples/sheetcards-examples.xlsx
@@ -1245,7 +1245,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t xml:space="preserve">今日很热。</t>
+          <t xml:space="preserve">明天是我的生日。</t>
         </is>
       </c>
     </row>
@@ -5269,7 +5269,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The last letter is a hamza, written on a seat here.</t>
+          <t xml:space="preserve">The last letter is a hamza, standing alone on the line.</t>
         </is>
       </c>
     </row>
@@ -8143,12 +8143,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">the mountain</t>
+          <t xml:space="preserve">the road</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ngọn núi</t>
+          <t xml:space="preserve">con đường</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">

</xml_diff>

<commit_message>
Example workbook: subdeck= columns, no retired keys, every key shown
Sheets that used SUBDECK n headers name their levels (Topic, Level, Language,
Word class) and say subdeck=n; sheet 15's deck tree is unchanged, checked row
by row. rtl, sort, vertical and the deck-wide align/speed are gone from every
sheet, and a font=sc/jp that tts now implies is dropped (templates render
byte-identical). test_examples expects font, type=nc, math and code; a new
real-Anki test imports sheet 15's old SUBDECK package, reviews a card, then
the converted one with Merge note types: same subdecks, progress kept.
</commit_message>
<xml_diff>
--- a/examples/sheetcards-examples.xlsx
+++ b/examples/sheetcards-examples.xlsx
@@ -24,7 +24,7 @@
     <sheet name="20 Video lesson (bài video)" sheetId="20" r:id="rId20"/>
     <sheet name="21 Formulas &amp; code (công thức)" sheetId="21" r:id="rId21"/>
     <sheet name="22 Arabic (phải sang trái)" sheetId="22" r:id="rId22"/>
-    <sheet name="23 Vertical text (viết dọc)" sheetId="23" r:id="rId23"/>
+    <sheet name="23 Haiku (thơ haiku)" sheetId="23" r:id="rId23"/>
     <sheet name="24 Korean (tiếng Hàn)" sheetId="24" r:id="rId24"/>
     <sheet name="25 Traditional (chữ phồn thể)" sheetId="25" r:id="rId25"/>
     <sheet name="26 Shell commands (dòng lệnh)" sheetId="26" r:id="rId26"/>
@@ -221,12 +221,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#config speed=0.9</t>
+          <t xml:space="preserve">#config</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">size=34; tts=en_US; voices=Samantha,Microsoft Zira</t>
+          <t xml:space="preserve">size=34; tts=en_US; voices=Samantha,Microsoft Zira; speed=0.9</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -479,7 +479,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">side=back; size=90; type; tts=zh_CN; font=sc; sort</t>
+          <t xml:space="preserve">side=back; size=90; type; tts=zh_CN</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1558,7 +1558,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUBDECK 1</t>
+          <t xml:space="preserve">Level</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1596,6 +1596,11 @@
       <c r="A2" t="inlineStr">
         <is>
           <t xml:space="preserve">#config</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subdeck=1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2529,17 +2534,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUBDECK 1</t>
+          <t xml:space="preserve">Language</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUBDECK 2</t>
+          <t xml:space="preserve">Level</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUBDECK 3</t>
+          <t xml:space="preserve">Word class</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -2574,9 +2579,24 @@
           <t xml:space="preserve">#config theme=sakura</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subdeck=1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subdeck=2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">subdeck=3</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">size=44; bold; tts=en_US; sort</t>
+          <t xml:space="preserve">size=44; bold; tts=en_US</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4433,12 +4453,12 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUBDECK 1</t>
+          <t xml:space="preserve">Topic</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUBDECK 2</t>
+          <t xml:space="preserve">Subtopic</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -4460,49 +4480,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">s01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">#config</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Geography</t>
+          <t xml:space="preserve">subdeck=1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capitals</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">europe, capitals</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Capital of Portugal?</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lisbon</t>
+          <t xml:space="preserve">subdeck=2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">s02</t>
+          <t xml:space="preserve">s01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">x</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -4517,29 +4517,29 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">asia; capitals</t>
+          <t xml:space="preserve">europe, capitals</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capital of Vietnam?</t>
+          <t xml:space="preserve">Capital of Portugal?</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hanoi</t>
+          <t xml:space="preserve">Lisbon</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">s03</t>
+          <t xml:space="preserve">s02</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">x</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4549,34 +4549,34 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rivers</t>
+          <t xml:space="preserve">Capitals</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivers</t>
+          <t xml:space="preserve">asia; capitals</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Longest river in Asia?</t>
+          <t xml:space="preserve">Capital of Vietnam?</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Yangtze</t>
+          <t xml:space="preserve">Hanoi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">s04</t>
+          <t xml:space="preserve">s03</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRUE</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4591,133 +4591,170 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">rivers, europe</t>
+          <t xml:space="preserve">rivers</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Which river flows through Paris?</t>
+          <t xml:space="preserve">Longest river in Asia?</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Seine</t>
+          <t xml:space="preserve">The Yangtze</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">s05</t>
+          <t xml:space="preserve">s04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">✓</t>
+          <t xml:space="preserve">TRUE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">History</t>
+          <t xml:space="preserve">Geography</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rivers</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">history</t>
+          <t xml:space="preserve">rivers, europe</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Who was the first Ming emperor?</t>
+          <t xml:space="preserve">Which river flows through Paris?</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Hongwu Emperor</t>
+          <t xml:space="preserve">The Seine</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">s06</t>
+          <t xml:space="preserve">s05</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">yes</t>
+          <t xml:space="preserve">✓</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">History</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">history</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Where does a row with both SUBDECK cells empty go?</t>
+          <t xml:space="preserve">Who was the first Ming emperor?</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Into 'Unsorted'. A sheet that sorts its rows has somewhere for the ones it did not sort.</t>
+          <t xml:space="preserve">The Hongwu Emperor</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">s07</t>
+          <t xml:space="preserve">s06</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">no</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Geography</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Capitals</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">capitals</t>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">This row is switched off.</t>
+          <t xml:space="preserve">Where does a row with both Topic and Subtopic empty go?</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve">It is never written to Anki.</t>
+          <t xml:space="preserve">Into 'Unsorted'. A sheet that sorts its rows has somewhere for the ones it did not sort.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">s07</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Geography</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Capitals</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">capitals</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">This row is switched off.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">It is never written to Anki.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t xml:space="preserve">s08</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t xml:space="preserve">History</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t xml:space="preserve">history</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t xml:space="preserve">An empty SYNC cell is off too.</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t xml:space="preserve">Same as 'no'.</t>
         </is>
@@ -4917,7 +4954,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">side=front; size=24; sort</t>
+          <t xml:space="preserve">side=front; size=24</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -5173,7 +5210,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">rtl; size=44; font=serif; sort</t>
+          <t xml:space="preserve">size=44; font=serif</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5391,7 +5428,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">vertical; font=jp; size=30; sort</t>
+          <t xml:space="preserve">size=30; tts=ja_JP</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5557,7 +5594,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">font=kr; size=44; tts=ko_KR; sort</t>
+          <t xml:space="preserve">size=44; tts=ko_KR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -5834,7 +5871,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">font=tc; size=48; tts=zh_TW; sort</t>
+          <t xml:space="preserve">size=48; tts=zh_TW</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -6116,7 +6153,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">side=front; size=24; sort</t>
+          <t xml:space="preserve">side=front; size=24</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -6388,7 +6425,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">side=front; size=22; sort</t>
+          <t xml:space="preserve">side=front; size=22</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -6578,7 +6615,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">side=front; size=22; sort</t>
+          <t xml:space="preserve">side=front; size=22</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -6826,7 +6863,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">cloze; size=26; tts=en_US; sort</t>
+          <t xml:space="preserve">cloze; size=26; tts=en_US</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -7041,27 +7078,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">#config align=left</t>
+          <t xml:space="preserve">#config</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">size=48px; bold</t>
+          <t xml:space="preserve">size=48px; bold; align=left</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">side=front; size=22; color=accent</t>
+          <t xml:space="preserve">side=front; size=22; color=accent; align=left</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">size=26; color=#c2410c</t>
+          <t xml:space="preserve">size=26; color=#c2410c; align=left</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">size=16; color=muted; italic; label=Example</t>
+          <t xml:space="preserve">size=16; color=muted; italic; label; align=left</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -7349,7 +7386,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">side=front; size=40; tts=de_DE; sort</t>
+          <t xml:space="preserve">side=front; size=40; tts=de_DE</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -7629,7 +7666,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">size=28; sort</t>
+          <t xml:space="preserve">size=28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>